<commit_message>
Add Wt (F)/Wt (R) columns to the print template
design.xlsx had no placeholder cells for the WEIGHTFRONT/WEIGHTREAR
tokens layout_constants.py already defines, so front/rear weight
values (populated by both the Canvas and Meyer parsers) never had
anywhere to display or export to. Relocated the existing Pick (R)
row pair down and inserted Wt (F)/Wt (R) between Pick (F) and Pick
(R), matching METADATA_TOKEN_ORDER physically as well as on-screen --
verified against both scan_template_layout() and a real
write_master_workbook() export.
</commit_message>
<xml_diff>
--- a/design.xlsx
+++ b/design.xlsx
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="B1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="2" max="2"/>
@@ -791,7 +791,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="D7" s="26" t="inlineStr">
         <is>
@@ -1351,14 +1350,42 @@
       </c>
       <c r="K24" s="15" t="inlineStr">
         <is>
-          <t>Pick (R)</t>
+          <t>Wt (F)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="K25" s="17" t="inlineStr">
         <is>
+          <t>SEC1_WEIGHTFRONT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>Pick (R)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="K27" s="17" t="inlineStr">
+        <is>
           <t>SEC1_PICKREAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>Wt (R)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>SEC1_WEIGHTREAR</t>
         </is>
       </c>
     </row>

</xml_diff>